<commit_message>
Sepatrate columns for Olga's and Italo's ana;lysis, proposal and model
</commit_message>
<xml_diff>
--- a/SIMAP-Model-Analysis/Olga's and Italo's proposal.xlsx
+++ b/SIMAP-Model-Analysis/Olga's and Italo's proposal.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\projects\ietf\Misc\SIMAP-Model-Analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B8F0718D-A808-4248-9268-5E18C3CD54ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E56B5DC-FDBE-4975-84C2-7B1B2C1D91F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-1545" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="48">
   <si>
     <t>Requirement</t>
   </si>
@@ -47,13 +47,7 @@
     <t>Olga's proposal</t>
   </si>
   <si>
-    <t>Analysis Summary</t>
-  </si>
-  <si>
     <t>REQ-BASIC-MODEL-SUPPORT</t>
-  </si>
-  <si>
-    <t>Model Suggested</t>
   </si>
   <si>
     <r>
@@ -258,26 +252,73 @@
 2.We analyzed what extensions are needed for the SIMAP model based on RFC8345 to support path computation and identified that the following is needed for supporting relation for links: order, preference, weight</t>
   </si>
   <si>
-    <t>Option 3: Generic way for any extensions via extensions attributes (via anydata to support completely unstructured data)
-Apply this grouping to every major entity in the topology model and in supporting relations.
-     grouping simap-common {
-       description "A reusable set of optional extensions for network,
-                    node, termination point and link";
-       :
-       :
-       anydata extension {
-         description
-           "The extension point for any other meta info or data or any
-           unknown extensions. Proposed solution for SIMAP requirement
-           REQ-EXTENSIBLE. Any additional info that is topologically
-           significant can also be added this way for requirement
-           REQ-SEMANTIC or REQ-PROPERTIES.";
-       }
-     }</t>
-  </si>
-  <si>
     <t>No model changes mandatory to to basic navigation for current tunnels/paths, but additional semantics required to understand supporting relations meaning for multiple tunnels and paths configured/used. 
 We identified order, preference and weight as important meta data that needs to be added - proposal in REQ-SEMANTIC.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Although we identified the attributes needed for this case, some other attributes may be needed based on other use cases. 
+Therefore there are 2 approaches: either add exact attributes to the supporting relation via augmentation or reuse the generic approach for REQ-EXTENSION to enable any extension.
+There are pros and cons of each approach, and the target model can support all 3. For attributes that we know based on hackathons and product experience, we can use Option1, for any future ones we can allow extensions via Option 2/3.
+Alternatively, we can go with Option 2 for any RFC8345 attribute extensions, with additional fields that can identify all required meta data for the attributes. </t>
+  </si>
+  <si>
+    <t>Our requirement from the modelling exercise / PoCs / Hackathon is that we had some TPs at higher layers that do not have supporting relation to TPs at the lower layer and the only way to be able to navigate supporting dependencies top to bottom (or for assurance bottom to top) was to add supporting relation to node at the lower layer. Examples: loopback is at Layer 3, but does not have Layer 2 or Physical TP for supporting. We also have in PoC one type of SID (that we modelled as TPs) at SRv6 layer that did not have any TPs as supporting, so we needed to build relation to the Node at the layer below.
+There was also requirement that Italo had to have supporting between a node and a network.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Augment RFC8345 nodes and termination-points to support the new supporting relations.</t>
+  </si>
+  <si>
+    <t>augment "/nw:networks/nw:network/nw:node/nt:termination-point" {
+  container supporting-node {
+    leaf network-ref {
+      type leafref {
+        path "/nw:networks/nw:network/nw:network-id";
+      }
+    }
+    leaf node-ref {
+      type leafref {
+        path "/nw:networks/nw:network[nw:network-id=current()/../network-ref]"
+           + "/nw:node/nw:node-id";
+      }
+    }
+    description
+      "Identifies the specific node that supports this termination point.";
+  }
+}</t>
+  </si>
+  <si>
+    <t>Italo's proposal</t>
+  </si>
+  <si>
+    <t>Re-use (a subset of) RFC8795 to model the underlay path of a link and link bundling</t>
+  </si>
+  <si>
+    <t>REF8795 inherits this capability from RFC8345 so it seems both approaches are aligned here
+Not clear how tunnel and path can be modelled as sub-layers ...</t>
+  </si>
+  <si>
+    <t>Re-use (a subset of) RFC8795 to model the underlay path of a link.
+This relationship is recursive and can be used to navigate across multiple layer down to the whole layer hierarchy until the lowest layer.
+The models under definition in IVY WG can be used to associate the link in the lowest level of the hierarchy with the cable: these models are compatible with and complimentary to RFC8795.</t>
+  </si>
+  <si>
+    <t>Re-use (a subset of) RFC8795 to model the underlay path of a link and link bundling to represent the order of the links along the path, whether the path is a primary or secondary path and whether there are multiple parallel paths</t>
+  </si>
+  <si>
+    <t>Reuse the underlay-topology, defined in RFC8795, to model the case where a node is supported by a newtork
+More discussion is needed to better understand the use cases where a TP is supported by a node: the use cases mentioned are packet technology-specific.</t>
+  </si>
+  <si>
+    <t>Olga's Analysis Summary</t>
+  </si>
+  <si>
+    <t>Italo's Analysis Summary</t>
+  </si>
+  <si>
+    <t>We followed the RFC8345 approach and did the same in Hackathons and PoC for L2/L3/ISIS/OSPF/BGP/MPLS-TE/MPLS-LDP/SRv6/L3VPN. We modelled all layers, including tunnels and paths using the basic IETF approach. We identified some additional fields that are needed for supporting relations to add semantics, but we determined that all topological layers and entities can be modelled via the RFC8345 entities and relations and that these fields can be added via just adding fields to RFC8345 entities and relations.
+RFC8795 implements subset of TE entities by augmenting network, node, link, but introduces new entities outside of RFC8345 topology, without augmenting RFC8345 entities for: tunnel, tunnel tp, path, path element, connectivity matrix</t>
   </si>
   <si>
     <r>
@@ -327,9 +368,14 @@
 }
 </t>
     </r>
-  </si>
-  <si>
-    <t>Option 2: Generic way for any extensions via extensions attributes (via identityref)
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">
+Option 2: Generic way for any extensions via extensions attributes (via identityref)
 Apply this grouping to every major entity in the topology model and in supporting relations.
 grouping generic-attributes {
   list attribute {
@@ -351,164 +397,40 @@
 identity link-supporting-attribute-type {
   base attribute-type;
   description "Base identity for all link supporting attribute types";
-}</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Although we identified the attributes needed for this case, some other attributes may be needed based on other use cases. 
-Therefore there are 2 approaches: either add exact attributes to the supporting relation via augmentation or reuse the generic approach for REQ-EXTENSION to enable any extension.
-There are pros and cons of each approach, and the target model can support all 3. For attributes that we know based on hackathons and product experience, we can use Option1, for any future ones we can allow extensions via Option 2/3.
-Alternatively, we can go with Option 2 for any RFC8345 attribute extensions, with additional fields that can identify all required meta data for the attributes. </t>
-  </si>
-  <si>
-    <t>Our requirement from the modelling exercise / PoCs / Hackathon is that we had some TPs at higher layers that do not have supporting relation to TPs at the lower layer and the only way to be able to navigate supporting dependencies top to bottom (or for assurance bottom to top) was to add supporting relation to node at the lower layer. Examples: loopback is at Layer 3, but does not have Layer 2 or Physical TP for supporting. We also have in PoC one type of SID (that we modelled as TPs) at SRv6 layer that did not have any TPs as supporting, so we needed to build relation to the Node at the layer below.
-There was also requirement that Italo had to have supporting between a node and a network.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Augment RFC8345 nodes and termination-points to support the new supporting relations.</t>
-  </si>
-  <si>
-    <t>augment "/nw:networks/nw:network/nw:node/nt:termination-point" {
-  container supporting-node {
-    leaf network-ref {
-      type leafref {
-        path "/nw:networks/nw:network/nw:network-id";
-      }
-    }
-    leaf node-ref {
-      type leafref {
-        path "/nw:networks/nw:network[nw:network-id=current()/../network-ref]"
-           + "/nw:node/nw:node-id";
-      }
-    }
-    description
-      "Identifies the specific node that supports this termination point.";
-  }
-}</t>
-  </si>
-  <si>
-    <t>Italo's proposal</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">We followed the RFC8345 approach and did the same in Hackathons and PoC for L2/L3/ISIS/OSPF/BGP/MPLS-TE/MPLS-LDP/SRv6/L3VPN. We modelled all layers, including tunnels and paths using the basic IETF approach. We identified some additional fields that are needed for supporting relations to add semantics, but we determined that all topological layers and entities can be modelled via the RFC8345 entities and relations and that these fields can be added via just adding fields to RFC8345 entities and relations.
-RFC8795 </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">implements subset of TE entities by augmenting </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">augments </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">network, node, link, but introduces new </t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">entities outside of RFC8345 topology, without augmenting RFC8345 entities for: tunnel, tunnel tp, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">bundled-link, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">path, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">and </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>path element</t>
-    </r>
-    <r>
-      <rPr>
-        <strike/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>, connectivity matrix</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF00B050"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> entities to model the underlay paths of a link to address some issues identified with the use of the supporting links, as defined in RFC8345:
+}
+Option 3: Generic way for any extensions via extensions attributes (via anydata to support completely unstructured data)
+Apply this grouping to every major entity in the topology model and in supporting relations.
+     grouping simap-common {
+       description "A reusable set of optional extensions for network,
+                    node, termination point and link";
+       :
+       :
+       anydata extension {
+         description
+           "The extension point for any other meta info or data or any
+           unknown extensions. Proposed solution for SIMAP requirement
+           REQ-EXTENSIBLE. Any additional info that is topologically
+           significant can also be added this way for requirement
+           REQ-SEMANTIC or REQ-PROPERTIES.";
+       }
+     }
+</t>
+    </r>
+  </si>
+  <si>
+    <t>Olga's Model Suggested</t>
+  </si>
+  <si>
+    <t>Italo's Model Suggested</t>
+  </si>
+  <si>
+    <t>RFC8795 augments network, node, link, but introduces new entities  bundled-link, path, and path element  to model the underlay paths of a link to address some issues identified with the use of the supporting links, as defined in RFC8345:
 - when a link L is supported by two links L1 and L2, it is not clear whether link L is a bundle link, with links L1 and L2 being its component links, or is an overlay link, with links L1 and L2 being the two links along its underlay path
 -a path is a ordered list while the supporting links is unordered: in other words, is the underlay path L1-L2 or L2-L1?
 - if the underlay path is protected, it is not clear which link belongs to the primary and which link belong to the backup path, e.g., is link L protected with L1 being the only path on the primary underly path and L2 the only path on the backup underly path or is link L1 unprotected with links L1 and L2 being the two links on the only primary underlay path?
 - if there are multiple backup paths, it is not clear which link belongs to which backup path
 - if the protection is segmented, we need to represent the PLR and merge nodes: so the path elements could be links or nodes
 It is also worth noting that the path-element entity is extensible and this extensibility has been beneficial to model technology-specific path elements (e.g,. transponders or 3R regenerators) and their relative order along the path</t>
-    </r>
-  </si>
-  <si>
-    <t>Re-use (a subset of) RFC8795 to model the underlay path of a link and link bundling</t>
-  </si>
-  <si>
-    <t>REF8795 inherits this capability from RFC8345 so it seems both approaches are aligned here
-Not clear how tunnel and path can be modelled as sub-layers ...</t>
-  </si>
-  <si>
-    <t>Re-use (a subset of) RFC8795 to model the underlay path of a link.
-This relationship is recursive and can be used to navigate across multiple layer down to the whole layer hierarchy until the lowest layer.
-The models under definition in IVY WG can be used to associate the link in the lowest level of the hierarchy with the cable: these models are compatible with and complimentary to RFC8795.</t>
-  </si>
-  <si>
-    <t>Re-use (a subset of) RFC8795 to model the underlay path of a link and link bundling to represent the order of the links along the path, whether the path is a primary or secondary path and whether there are multiple parallel paths</t>
-  </si>
-  <si>
-    <t>Reuse the underlay-topology, defined in RFC8795, to model the case where a node is supported by a newtork
-More discussion is needed to better understand the use cases where a TP is supported by a node: the use cases mentioned are packet technology-specific.</t>
   </si>
 </sst>
 </file>
@@ -539,25 +461,36 @@
       <family val="2"/>
     </font>
     <font>
-      <strike/>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
+      <color rgb="FF00B050"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FF00B050"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -589,7 +522,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -602,23 +535,35 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -958,254 +903,277 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:K11"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="2" max="2" width="28.9140625" customWidth="1"/>
     <col min="3" max="3" width="35.83203125" customWidth="1"/>
-    <col min="4" max="5" width="49.83203125" customWidth="1"/>
-    <col min="6" max="6" width="32.33203125" customWidth="1"/>
-    <col min="7" max="7" width="32.33203125" style="9" customWidth="1"/>
-    <col min="8" max="8" width="73.33203125" customWidth="1"/>
-    <col min="9" max="9" width="81.9140625" customWidth="1"/>
-    <col min="10" max="10" width="79.1640625" customWidth="1"/>
+    <col min="4" max="6" width="49.83203125" customWidth="1"/>
+    <col min="7" max="7" width="32.33203125" customWidth="1"/>
+    <col min="8" max="8" width="32.33203125" style="6" customWidth="1"/>
+    <col min="9" max="9" width="63.08203125" customWidth="1"/>
+    <col min="10" max="10" width="51.5" customWidth="1"/>
+    <col min="11" max="11" width="50.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10">
+    <row r="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
+      <c r="E1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="11" t="s">
+        <v>42</v>
+      </c>
+      <c r="G1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="G1" s="7" t="s">
-        <v>40</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>5</v>
+      <c r="H1" s="9" t="s">
+        <v>35</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="J1" s="11" t="s">
+        <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:10">
+    <row r="2" spans="1:11">
       <c r="A2" s="1"/>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
+      <c r="E2" s="7"/>
+      <c r="F2" s="11"/>
       <c r="G2" s="7"/>
-      <c r="H2" s="1"/>
+      <c r="H2" s="9"/>
+      <c r="I2" s="7"/>
+      <c r="J2" s="11"/>
     </row>
-    <row r="3" spans="1:10" ht="409.5" customHeight="1">
+    <row r="3" spans="1:11" ht="409.5" customHeight="1">
       <c r="A3" s="1">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>25</v>
+      <c r="E3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="F3" s="12" t="s">
+        <v>47</v>
       </c>
       <c r="G3" s="8" t="s">
-        <v>42</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>7</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="H3" s="10" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" s="11"/>
     </row>
-    <row r="4" spans="1:10" ht="321.5" customHeight="1">
+    <row r="4" spans="1:11" ht="321.5" customHeight="1">
       <c r="A4" s="1">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="E4" s="8" t="s">
         <v>24</v>
       </c>
-      <c r="E4" s="3" t="s">
+      <c r="F4" s="12"/>
+      <c r="G4" s="8" t="s">
         <v>26</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="G4" s="8" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>27</v>
-      </c>
+      <c r="H4" s="10" t="s">
+        <v>37</v>
+      </c>
+      <c r="I4" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="J4" s="11"/>
     </row>
-    <row r="5" spans="1:10" ht="165" customHeight="1">
+    <row r="5" spans="1:11" ht="165" customHeight="1">
       <c r="A5" s="1">
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="D5" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="F5" s="3" t="s">
+      <c r="E5" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="F5" s="12"/>
+      <c r="G5" s="8" t="s">
+        <v>28</v>
+      </c>
+      <c r="H5" s="10" t="s">
+        <v>38</v>
+      </c>
+      <c r="I5" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="8" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>33</v>
-      </c>
+      <c r="J5" s="11"/>
     </row>
-    <row r="6" spans="1:10" ht="409.5" customHeight="1">
+    <row r="6" spans="1:11" ht="409.5" customHeight="1">
       <c r="A6" s="1">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="D6" s="3" t="s">
-        <v>21</v>
-      </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="F6" s="12"/>
+      <c r="G6" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="F6" s="3" t="s">
-        <v>36</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="I6" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="J6" s="5" t="s">
-        <v>32</v>
-      </c>
+      <c r="H6" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="J6" s="12"/>
+      <c r="K6" s="4"/>
     </row>
-    <row r="7" spans="1:10" ht="196">
+    <row r="7" spans="1:11" ht="196">
       <c r="A7" s="1">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>37</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>38</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="F7" s="12"/>
       <c r="G7" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" s="6" t="s">
-        <v>39</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="H7" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="J7" s="11"/>
     </row>
-    <row r="8" spans="1:10">
+    <row r="8" spans="1:11">
       <c r="A8" s="1">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D8" s="1"/>
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="1"/>
+      <c r="G8" s="1"/>
+      <c r="H8" s="5"/>
+      <c r="I8" s="1"/>
+      <c r="J8" s="1"/>
     </row>
-    <row r="9" spans="1:10">
+    <row r="9" spans="1:11">
       <c r="A9" s="1">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="D9" s="1"/>
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="1"/>
+      <c r="G9" s="1"/>
+      <c r="H9" s="5"/>
+      <c r="I9" s="1"/>
+      <c r="J9" s="1"/>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:11">
       <c r="A10" s="1">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D10" s="1"/>
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="1"/>
+      <c r="G10" s="1"/>
+      <c r="H10" s="5"/>
+      <c r="I10" s="1"/>
+      <c r="J10" s="1"/>
     </row>
-    <row r="11" spans="1:10">
+    <row r="11" spans="1:11">
       <c r="A11" s="1">
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="1"/>
+      <c r="G11" s="1"/>
+      <c r="H11" s="5"/>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="0" type="noConversion"/>

</xml_diff>